<commit_message>
feat: include_section 예제 확장 - 섹션 내부 for 루프 추가
- 섹션 컴포넌트 내에서 for 루프 사용 예제 추가
- 중첩 데이터 context 전달 테스트 (order.items)
- 버전 0.5.1
</commit_message>
<xml_diff>
--- a/examples/include_section_output.xlsx
+++ b/examples/include_section_output.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -495,58 +495,148 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>주문 #1002</t>
+          <t xml:space="preserve">  - 프리미엄 앨범</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>이영희</t>
+          <t>2개</t>
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>35000</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>⭐ VIP 주문 #1003</t>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - 포토카드 세트</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>박지민</t>
+          <t>1개</t>
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>280000</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>주문 #1002</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>이영희</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - 일반 앨범</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>1개</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>⭐ VIP 주문 #1003</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>박지민</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>280000</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - 한정판 앨범</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>1개</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - 굿즈 패키지</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2개</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>65000</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>주문 #1004</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>최수진</t>
         </is>
       </c>
-      <c r="C8" s="4" t="n">
+      <c r="C13" s="4" t="n">
         <v>42000</v>
       </c>
     </row>
-    <row r="9"/>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - 포스터 세트</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>3개</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>14000</v>
+      </c>
+    </row>
+    <row r="15"/>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>총 4건의 주문</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>문의: support@makestar.com</t>
         </is>
@@ -563,7 +653,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -628,67 +718,129 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>{# enddefine_section #}</t>
-        </is>
-      </c>
-    </row>
-    <row r="10"/>
+          <t>{% for item in order.items %}</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - {{ item.name }}</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>{{ item.qty }}개</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>{{ item.price }}</t>
+        </is>
+      </c>
+    </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>{# define_section:일반_주문 #}</t>
+          <t>{% endfor %}</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>주문 #{{ order.id }}</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>{{ order.customer }}</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>{{ order.amount }}</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
           <t>{# enddefine_section #}</t>
         </is>
       </c>
     </row>
-    <row r="14"/>
+    <row r="13"/>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>{# define_section:일반_주문 #}</t>
+        </is>
+      </c>
+    </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>{# define_section:푸터 #}</t>
-        </is>
-      </c>
-    </row>
-    <row r="16"/>
+          <t>주문 #{{ order.id }}</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>{{ order.customer }}</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>{{ order.amount }}</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>{% for item in order.items %}</t>
+        </is>
+      </c>
+    </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>총 {{ orders|length }}건의 주문</t>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - {{ item.name }}</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>{{ item.qty }}개</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>{{ item.price }}</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>문의: {{ contact_email }}</t>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>{% endfor %}</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
+        <is>
+          <t>{# enddefine_section #}</t>
+        </is>
+      </c>
+    </row>
+    <row r="20"/>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>{# define_section:푸터 #}</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>총 {{ orders|length }}건의 주문</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>문의: {{ contact_email }}</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
         <is>
           <t>{# enddefine_section #}</t>
         </is>

</xml_diff>